<commit_message>
Rename the old file to a new one
</commit_message>
<xml_diff>
--- a/DAY_02/Day2-Exercise.xlsx
+++ b/DAY_02/Day2-Exercise.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a96f5c588f37a5dc/Desktop/MJ/TESDA/DAY_02/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{FBFCA139-48A8-4BE2-A2EF-FBEC8430D1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9882D7D7-CAED-48E7-9381-26A8D828D942}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{FBFCA139-48A8-4BE2-A2EF-FBEC8430D1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D16B5C2-88C4-42A2-96A9-128216191C66}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{9F0A8D4D-891B-4EB3-B8AC-C5A108C41033}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
   <si>
     <t>Student_1</t>
   </si>
@@ -143,6 +143,15 @@
   </si>
   <si>
     <t>Score</t>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>Summation</t>
+  </si>
+  <si>
+    <t>Average</t>
   </si>
 </sst>
 </file>
@@ -164,15 +173,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -180,11 +201,121 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -194,6 +325,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -226,7 +381,7 @@
     <tableColumn id="1" xr3:uid="{9DB1914E-74F0-4F40-9919-14CC0F73DBB6}" name="Student" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{4E5F59EC-F60A-4CAC-A078-22D18CEE9341}" name="Score" dataDxfId="0"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -730,47 +885,74 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{859B544E-5201-49FC-BE19-9E6FD9413988}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="2" customWidth="1"/>
     <col min="2" max="2" width="13.85546875" style="2" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="2"/>
+    <col min="3" max="3" width="9.140625" style="2"/>
+    <col min="4" max="4" width="11.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D1" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="11"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B2" s="1">
         <v>85</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="4">
+        <f>SUM(Table1[Score])</f>
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B3" s="1">
         <v>92</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="5">
+        <f>COUNT(Table1[Score])</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B4" s="1">
         <v>78</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D4" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="6">
+        <f>AVERAGE(Table1[Score])</f>
+        <v>86.6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>32</v>
       </c>
@@ -778,7 +960,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>33</v>
       </c>
@@ -787,6 +969,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D1:E1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>